<commit_message>
Enhance debugging and validation.
</commit_message>
<xml_diff>
--- a/instruction_data/templates/nature_lookup.xlsx
+++ b/instruction_data/templates/nature_lookup.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/raw_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{209E2443-AC32-4149-9E33-E84E3CE31CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FDFC33F-7275-F84D-83FD-59F6B3609D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{7F521D3B-2E69-8A47-969D-D626CAA8171E}"/>
   </bookViews>
@@ -88,30 +88,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="179">
   <si>
     <t xml:space="preserve">Organisational capacity building </t>
-  </si>
-  <si>
-    <t>SI,</t>
-  </si>
-  <si>
-    <t>PIT</t>
-  </si>
-  <si>
-    <t>bonus</t>
-  </si>
-  <si>
-    <t>salary</t>
-  </si>
-  <si>
-    <t>reimbursement</t>
-  </si>
-  <si>
-    <t>advance by cash</t>
-  </si>
-  <si>
-    <t>advance</t>
   </si>
   <si>
     <t>1500VN</t>
@@ -1140,52 +1119,52 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="19" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="27" x14ac:dyDescent="0.2">
       <c r="B5" s="18" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B6" s="15" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -1195,16 +1174,16 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B7" s="15" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
@@ -1214,16 +1193,16 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B8" s="15" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
@@ -1233,16 +1212,16 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B9" s="15" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
@@ -1252,16 +1231,16 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B10" s="15" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
@@ -1271,16 +1250,16 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" s="15" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
@@ -1290,16 +1269,16 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B12" s="15" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -1309,16 +1288,16 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B13" s="15" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
@@ -1328,16 +1307,16 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B14" s="15" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -1347,16 +1326,16 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B15" s="15" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
@@ -1366,16 +1345,16 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B16" s="15" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
@@ -1385,16 +1364,16 @@
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B17" s="15" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
@@ -1404,16 +1383,16 @@
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B18" s="15" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
@@ -1423,16 +1402,16 @@
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B19" s="15" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -1442,16 +1421,16 @@
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B20" s="15" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -1461,16 +1440,16 @@
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B21" s="15" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -1480,16 +1459,16 @@
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B22" s="15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
@@ -1499,16 +1478,16 @@
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B23" s="15" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -1518,16 +1497,16 @@
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B24" s="15" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -1537,16 +1516,16 @@
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B25" s="15" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
@@ -1556,16 +1535,16 @@
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B26" s="15" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
@@ -1575,16 +1554,16 @@
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B27" s="15" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
@@ -1594,16 +1573,16 @@
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B28" s="15" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F28" s="12"/>
       <c r="G28" s="12"/>
@@ -1613,16 +1592,16 @@
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B29" s="15" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F29" s="12"/>
       <c r="G29" s="12"/>
@@ -1632,16 +1611,16 @@
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B30" s="15" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
@@ -1651,16 +1630,16 @@
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B31" s="15" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
@@ -1670,16 +1649,16 @@
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B32" s="15" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F32" s="12"/>
       <c r="G32" s="12"/>
@@ -1689,16 +1668,16 @@
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B33" s="15" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
@@ -1708,16 +1687,16 @@
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B34" s="15" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
@@ -1727,16 +1706,16 @@
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B35" s="15" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -1746,16 +1725,16 @@
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B36" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
@@ -1765,16 +1744,16 @@
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B37" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
@@ -1784,16 +1763,16 @@
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B38" s="15" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F38" s="12"/>
       <c r="G38" s="12"/>
@@ -1803,16 +1782,16 @@
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B39" s="15" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
@@ -1822,16 +1801,16 @@
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B40" s="15" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
@@ -1841,16 +1820,16 @@
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B41" s="15" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
@@ -1860,843 +1839,843 @@
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B42" s="15" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F42" s="12"/>
       <c r="G42" s="12"/>
       <c r="H42" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B43" s="15" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
       <c r="H43" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" s="15" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
       <c r="H44" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B45" s="15" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
       <c r="H45" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B46" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
       <c r="H46" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B47" s="15" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
       <c r="H47" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B48" s="15" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
       <c r="H48" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B49" s="15" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
       <c r="H49" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B50" s="15" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F50" s="12"/>
       <c r="G50" s="12"/>
       <c r="H50" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B51" s="15" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
       <c r="H51" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B52" s="15" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F52" s="12"/>
       <c r="G52" s="12"/>
       <c r="H52" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B53" s="15" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
       <c r="H53" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B54" s="15" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
       <c r="H54" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B55" s="15" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
       <c r="H55" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="56" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B56" s="15" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
       <c r="H56" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B57" s="15" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
       <c r="H57" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B58" s="15" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
       <c r="H58" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B59" s="15" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
       <c r="H59" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B60" s="15" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F60" s="12"/>
       <c r="G60" s="12"/>
       <c r="H60" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B61" s="15" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
       <c r="H61" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B62" s="15" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F62" s="12"/>
       <c r="G62" s="12"/>
       <c r="H62" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B63" s="15" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C63" s="13" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E63" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F63" s="12"/>
       <c r="G63" s="12"/>
       <c r="H63" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B64" s="15" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E64" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F64" s="12"/>
       <c r="G64" s="12"/>
       <c r="H64" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B65" s="15" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C65" s="13" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E65" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
       <c r="H65" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B66" s="15" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D66" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E66" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
       <c r="H66" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="67" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B67" s="15" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D67" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E67" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F67" s="12"/>
       <c r="G67" s="12"/>
       <c r="H67" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="68" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B68" s="15" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E68" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F68" s="12"/>
       <c r="G68" s="12"/>
       <c r="H68" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="69" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B69" s="15" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E69" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F69" s="12"/>
       <c r="G69" s="12"/>
       <c r="H69" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B70" s="15" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D70" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E70" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F70" s="12"/>
       <c r="G70" s="12"/>
       <c r="H70" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B71" s="15" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E71" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F71" s="12"/>
       <c r="G71" s="12"/>
       <c r="H71" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B72" s="15" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D72" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E72" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F72" s="12"/>
       <c r="G72" s="12"/>
       <c r="H72" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B73" s="15" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D73" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E73" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F73" s="12"/>
       <c r="G73" s="12"/>
       <c r="H73" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B74" s="15" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D74" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E74" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F74" s="12"/>
       <c r="G74" s="12"/>
       <c r="H74" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B75" s="15" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D75" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E75" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F75" s="12"/>
       <c r="G75" s="12"/>
       <c r="H75" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B76" s="15" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D76" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E76" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F76" s="12"/>
       <c r="G76" s="12"/>
       <c r="H76" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B77" s="15" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D77" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E77" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F77" s="12"/>
       <c r="G77" s="12"/>
       <c r="H77" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B78" s="15" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D78" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E78" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F78" s="12"/>
       <c r="G78" s="12"/>
       <c r="H78" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="79" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B79" s="15" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C79" s="13" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D79" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E79" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F79" s="12"/>
       <c r="G79" s="12"/>
       <c r="H79" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B80" s="15" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D80" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E80" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F80" s="12"/>
       <c r="G80" s="12"/>
       <c r="H80" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="81" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B81" s="15" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C81" s="13" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D81" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E81" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F81" s="12"/>
       <c r="G81" s="12"/>
       <c r="H81" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B82" s="15" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D82" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E82" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F82" s="12"/>
       <c r="G82" s="12"/>
       <c r="H82" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="83" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B83" s="15" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C83" s="13" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D83" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E83" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F83" s="12"/>
       <c r="G83" s="12"/>
       <c r="H83" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="84" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B84" s="15" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C84" s="13" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D84" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E84" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F84" s="12"/>
       <c r="G84" s="12"/>
       <c r="H84" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B85" s="15" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D85" s="12" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E85" s="12" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F85" s="12"/>
       <c r="G85" s="12"/>
       <c r="H85" s="9" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="86" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B86" s="14" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C86" s="13"/>
       <c r="D86" s="12"/>
@@ -2704,12 +2683,12 @@
       <c r="F86" s="12"/>
       <c r="G86" s="12"/>
       <c r="H86" s="1" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="87" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B87" s="14" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C87" s="13"/>
       <c r="D87" s="12"/>
@@ -2717,12 +2696,12 @@
       <c r="F87" s="12"/>
       <c r="G87" s="12"/>
       <c r="H87" s="1" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="88" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B88" s="14" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C88" s="13"/>
       <c r="D88" s="12"/>
@@ -2730,74 +2709,48 @@
       <c r="F88" s="12"/>
       <c r="G88" s="12"/>
       <c r="H88" s="1" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="89" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B89" s="2" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H89" s="1" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="90" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B90" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H90" s="11" t="s">
-        <v>6</v>
-      </c>
+      <c r="H90" s="11"/>
     </row>
     <row r="91" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B91" s="8" t="s">
-        <v>5</v>
-      </c>
+      <c r="B91" s="8"/>
       <c r="C91" s="7"/>
       <c r="E91" s="3"/>
-      <c r="H91" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="92" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B92" s="8" t="s">
-        <v>4</v>
-      </c>
+      <c r="B92" s="8"/>
       <c r="C92" s="7"/>
       <c r="E92" s="3"/>
-      <c r="H92" s="10" t="s">
-        <v>0</v>
-      </c>
+      <c r="H92" s="10"/>
     </row>
     <row r="93" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B93" s="8" t="s">
-        <v>3</v>
-      </c>
+      <c r="B93" s="8"/>
       <c r="C93" s="7"/>
       <c r="E93" s="3"/>
-      <c r="H93" s="9" t="s">
-        <v>0</v>
-      </c>
+      <c r="H93" s="9"/>
     </row>
     <row r="94" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B94" s="8" t="s">
-        <v>2</v>
-      </c>
+      <c r="B94" s="8"/>
       <c r="C94" s="7"/>
       <c r="E94" s="3"/>
-      <c r="H94" s="9" t="s">
-        <v>0</v>
-      </c>
+      <c r="H94" s="9"/>
     </row>
     <row r="95" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B95" s="8" t="s">
-        <v>1</v>
-      </c>
+      <c r="B95" s="8"/>
       <c r="C95" s="7"/>
       <c r="E95" s="3"/>
-      <c r="H95" s="9" t="s">
-        <v>0</v>
-      </c>
+      <c r="H95" s="9"/>
     </row>
     <row r="113" spans="2:8" ht="17" x14ac:dyDescent="0.2">
       <c r="B113" s="8"/>

</xml_diff>